<commit_message>
two more flexor tests
Looks like FlxTest04_20 should have been FlxTest05_01, etc.
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\melze\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDD150D4-4730-494D-96AC-EE7AD0BAEDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8F416346-DDA5-482A-BBD3-70514486EDB6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="26685" yWindow="-16200" windowWidth="14610" windowHeight="15585" firstSheet="13" activeTab="15" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
+    <workbookView xWindow="11910" yWindow="-16320" windowWidth="29040" windowHeight="15720" firstSheet="10" activeTab="15" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest10mm_1" sheetId="9" r:id="rId1"/>
@@ -294,7 +294,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="359" uniqueCount="81">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="354" uniqueCount="82">
   <si>
     <t>Test #</t>
   </si>
@@ -538,12 +538,15 @@
   <si>
     <t>^Collected by Moe &amp; Ben</t>
   </si>
+  <si>
+    <t>oooooo</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" mc:Ignorable="x14ac x16r2 xr xr9">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -585,12 +588,6 @@
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <sz val="9"/>
-      <color indexed="81"/>
-      <name val="Tahoma"/>
-      <charset val="1"/>
     </font>
   </fonts>
   <fills count="6">
@@ -4716,42 +4713,100 @@
               </a:ln>
               <a:effectLst/>
             </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
-          </c:trendline>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="linear"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
-          </c:trendline>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="19050" cap="rnd">
-                <a:solidFill>
-                  <a:schemeClr val="accent1"/>
-                </a:solidFill>
-                <a:prstDash val="sysDot"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
             <c:trendlineType val="poly"/>
             <c:order val="3"/>
             <c:dispRSqr val="1"/>
             <c:dispEq val="1"/>
             <c:trendlineLbl>
+              <c:layout>
+                <c:manualLayout>
+                  <c:x val="8.5337707786526634E-2"/>
+                  <c:y val="-0.46240994367386146"/>
+                </c:manualLayout>
+              </c:layout>
+              <c:tx>
+                <c:rich>
+                  <a:bodyPr rot="0" spcFirstLastPara="1" vertOverflow="ellipsis" vert="horz" wrap="square" anchor="ctr" anchorCtr="1"/>
+                  <a:lstStyle/>
+                  <a:p>
+                    <a:pPr>
+                      <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                        <a:latin typeface="+mn-lt"/>
+                        <a:ea typeface="+mn-ea"/>
+                        <a:cs typeface="+mn-cs"/>
+                      </a:defRPr>
+                    </a:pPr>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>y = 0.0001x</a:t>
+                    </a:r>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="30000">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>3</a:t>
+                    </a:r>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t> + 0.024x</a:t>
+                    </a:r>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="30000">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>2</a:t>
+                    </a:r>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t> + 0.9144x - 5.9593</a:t>
+                    </a:r>
+                    <a:br>
+                      <a:rPr lang="en-US" b="1" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                    </a:br>
+                    <a:r>
+                      <a:rPr lang="en-US" b="1" baseline="0">
+                        <a:solidFill>
+                          <a:schemeClr val="bg1"/>
+                        </a:solidFill>
+                      </a:rPr>
+                      <a:t>R² = 0.9885</a:t>
+                    </a:r>
+                    <a:endParaRPr lang="en-US" b="1">
+                      <a:solidFill>
+                        <a:schemeClr val="bg1"/>
+                      </a:solidFill>
+                    </a:endParaRPr>
+                  </a:p>
+                </c:rich>
+              </c:tx>
               <c:numFmt formatCode="General" sourceLinked="0"/>
               <c:spPr>
-                <a:noFill/>
+                <a:solidFill>
+                  <a:schemeClr val="tx1"/>
+                </a:solidFill>
                 <a:ln>
                   <a:noFill/>
                 </a:ln>
@@ -4764,10 +4819,7 @@
                   <a:pPr>
                     <a:defRPr sz="900" b="0" i="0" u="none" strike="noStrike" kern="1200" baseline="0">
                       <a:solidFill>
-                        <a:schemeClr val="tx1">
-                          <a:lumMod val="65000"/>
-                          <a:lumOff val="35000"/>
-                        </a:schemeClr>
+                        <a:schemeClr val="bg1"/>
                       </a:solidFill>
                       <a:latin typeface="+mn-lt"/>
                       <a:ea typeface="+mn-ea"/>
@@ -4809,6 +4861,36 @@
                 <c:pt idx="7">
                   <c:v>-24.202999999999999</c:v>
                 </c:pt>
+                <c:pt idx="8">
+                  <c:v>-25.6</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>-16</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>-20.6</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>-70.81</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>-63</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-53.6</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-39.280999999999999</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-29.6</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-16.3</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-10.199999999999999</c:v>
+                </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
@@ -4819,58 +4901,58 @@
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="22"/>
                 <c:pt idx="0">
-                  <c:v>-1.9089163300292105</c:v>
+                  <c:v>-1.9888446022622024</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>-4.0809375058192954</c:v>
+                  <c:v>-4.2527956349925518</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>-7.0574220518637798</c:v>
+                  <c:v>-7.3539886035989408</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>-10.09453321766197</c:v>
+                  <c:v>-10.527409285407064</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>-13.401234911810583</c:v>
+                  <c:v>-13.966402193997661</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>-14.847761858930939</c:v>
+                  <c:v>-15.473036951197667</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>-15.781617917093591</c:v>
+                  <c:v>-16.445267992387105</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>-16.386164614410578</c:v>
+                  <c:v>-17.07325998043143</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0</c:v>
+                  <c:v>-14.697192119709124</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0</c:v>
+                  <c:v>-15.358895091501429</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0</c:v>
+                  <c:v>-15.042937875530633</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>0</c:v>
+                  <c:v>-0.56433407059449248</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>0</c:v>
+                  <c:v>-2.4445410159422072</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>-5.2402184740344895</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>-10.95843156495609</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>-13.902438921694182</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
+                  <c:v>-16.846155017276384</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>-9.9320795468220986</c:v>
                 </c:pt>
                 <c:pt idx="18">
                   <c:v>0</c:v>
@@ -19099,24 +19181,24 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C83896A-0586-4C90-B5FD-474633C66A37}">
   <dimension ref="A1:AJ27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -19127,7 +19209,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -19136,7 +19218,7 @@
         <v>403.38</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -19144,7 +19226,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -19267,7 +19349,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -19332,7 +19414,7 @@
         <v>23.167999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -19397,7 +19479,7 @@
         <v>-123</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -19465,13 +19547,13 @@
         <v>84.4</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -19551,7 +19633,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -19577,7 +19659,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -19652,7 +19734,7 @@
         <v>264</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -19718,13 +19800,13 @@
         <v>37</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -19861,12 +19943,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="17" spans="3:24" x14ac:dyDescent="0.3">
       <c r="C17" t="s">
         <v>20</v>
       </c>
     </row>
-    <row r="18" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="18" spans="3:24" x14ac:dyDescent="0.3">
       <c r="C18">
         <f>C6+4.6262</f>
         <v>5.6261999999999999</v>
@@ -19904,7 +19986,7 @@
         <v>6.3061999999999996</v>
       </c>
     </row>
-    <row r="19" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="19" spans="3:24" x14ac:dyDescent="0.3">
       <c r="C19">
         <v>22.176200000000001</v>
       </c>
@@ -19933,12 +20015,12 @@
         <v>6.3061999999999996</v>
       </c>
     </row>
-    <row r="20" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="20" spans="3:24" x14ac:dyDescent="0.3">
       <c r="C20" t="s">
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="21" spans="3:24" x14ac:dyDescent="0.3">
       <c r="C21">
         <v>17.55</v>
       </c>
@@ -19967,7 +20049,7 @@
         <v>1.68</v>
       </c>
     </row>
-    <row r="22" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="22" spans="3:24" x14ac:dyDescent="0.3">
       <c r="T22">
         <v>480</v>
       </c>
@@ -19984,7 +20066,7 @@
         <v>405</v>
       </c>
     </row>
-    <row r="23" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="23" spans="3:24" x14ac:dyDescent="0.3">
       <c r="S23" t="s">
         <v>30</v>
       </c>
@@ -20009,7 +20091,7 @@
         <v>0.16666666666666666</v>
       </c>
     </row>
-    <row r="24" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="24" spans="3:24" x14ac:dyDescent="0.3">
       <c r="S24" t="s">
         <v>31</v>
       </c>
@@ -20034,7 +20116,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="3:24" x14ac:dyDescent="0.35">
+    <row r="27" spans="3:24" x14ac:dyDescent="0.3">
       <c r="S27" t="s">
         <v>32</v>
       </c>
@@ -20053,27 +20135,27 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EA3ACFF-8EC2-4AAF-BDC7-460D102A0BEE}">
   <dimension ref="A1:AE21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="12" max="12" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>62</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -20084,7 +20166,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -20100,7 +20182,7 @@
         <v>0.14749999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -20120,7 +20202,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -20212,7 +20294,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -20256,7 +20338,7 @@
         <v>20.7</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -20300,7 +20382,7 @@
         <v>-100</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>47</v>
       </c>
@@ -20344,7 +20426,7 @@
         <v>620</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -20391,7 +20473,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -20436,7 +20518,7 @@
         <v>382</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -20445,14 +20527,14 @@
       </c>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="16"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -20545,7 +20627,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -20590,14 +20672,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="14"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
@@ -20718,7 +20800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="L17" t="s">
         <v>55</v>
       </c>
@@ -20729,7 +20811,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
@@ -20745,27 +20827,27 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FE9CE551-57A5-4045-B5A9-E0D9326386C2}">
   <dimension ref="A1:AE27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="12" max="12" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -20776,7 +20858,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -20792,7 +20874,7 @@
         <v>0.15046296296296291</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -20804,7 +20886,7 @@
       </c>
       <c r="O4" s="3"/>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -20896,7 +20978,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -20943,7 +21025,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -20990,7 +21072,7 @@
         <v>-106.5</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>47</v>
       </c>
@@ -21037,7 +21119,7 @@
         <v>622</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -21087,7 +21169,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -21135,7 +21217,7 @@
         <v>403</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -21144,14 +21226,14 @@
       </c>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="16"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -21244,7 +21326,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -21292,14 +21374,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="14"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
@@ -21420,16 +21502,16 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="27" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B27" s="29" t="s">
         <v>67</v>
       </c>
@@ -21445,22 +21527,22 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{605CE535-3534-4BC1-886C-868F03FBDC68}">
   <dimension ref="A1:AK36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="39.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>61</v>
       </c>
       <c r="B1" s="3"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>71</v>
       </c>
@@ -21472,7 +21554,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>70</v>
       </c>
@@ -21489,7 +21571,7 @@
         <v>0.1490825688073395</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -21519,7 +21601,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>0</v>
@@ -21618,7 +21700,7 @@
       <c r="AJ5" s="10"/>
       <c r="AK5" s="10"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="5" t="s">
         <v>1</v>
@@ -21685,7 +21767,7 @@
         <v>0.40200000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>2</v>
@@ -21752,7 +21834,7 @@
         <v>31.442</v>
       </c>
     </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
         <v>47</v>
@@ -21819,7 +21901,7 @@
         <v>620.57899999999995</v>
       </c>
     </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -21902,74 +21984,74 @@
       <c r="AJ9" s="1"/>
       <c r="AK9" s="1"/>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
       </c>
       <c r="C10" s="30"/>
-      <c r="D10" s="33">
+      <c r="D10">
         <v>367</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10">
         <v>367</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10">
         <v>382</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10">
         <v>398</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10">
         <v>397</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10">
         <v>403</v>
       </c>
-      <c r="J10" s="33">
+      <c r="J10">
         <v>407</v>
       </c>
-      <c r="K10" s="33">
+      <c r="K10">
         <v>411</v>
       </c>
-      <c r="L10" s="33">
+      <c r="L10">
         <v>416</v>
       </c>
-      <c r="M10" s="33">
+      <c r="M10">
         <v>422</v>
       </c>
-      <c r="N10" s="33">
+      <c r="N10">
         <v>428</v>
       </c>
-      <c r="O10" s="33">
+      <c r="O10">
         <v>428</v>
       </c>
-      <c r="P10" s="33">
+      <c r="P10">
         <v>434</v>
       </c>
-      <c r="Q10" s="33">
+      <c r="Q10">
         <v>434</v>
       </c>
-      <c r="R10" s="33">
+      <c r="R10">
         <v>425</v>
       </c>
-      <c r="S10" s="33">
+      <c r="S10">
         <v>420</v>
       </c>
-      <c r="T10" s="33">
+      <c r="T10">
         <v>398</v>
       </c>
-      <c r="U10" s="33">
+      <c r="U10">
         <v>396</v>
       </c>
-      <c r="V10" s="33">
+      <c r="V10">
         <v>386</v>
       </c>
-      <c r="W10" s="33">
+      <c r="W10">
         <v>366</v>
       </c>
     </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -22012,14 +22094,14 @@
       <c r="AJ11" s="1"/>
       <c r="AK11" s="1"/>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="30"/>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -22112,7 +22194,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -22179,7 +22261,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
@@ -22220,7 +22302,7 @@
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="5" t="s">
         <v>6</v>
@@ -22342,91 +22424,91 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="29" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
     </row>
@@ -22440,24 +22522,24 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{09E5B9E9-F1B4-4DAB-B7CA-9BCB2303132C}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -22468,7 +22550,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -22477,7 +22559,7 @@
         <v>402.55</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -22485,7 +22567,7 @@
         <v>398</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -22608,7 +22690,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -22697,7 +22779,7 @@
         <v>30.405999999999999</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -22786,7 +22868,7 @@
         <v>19.5</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -22878,13 +22960,13 @@
         <v>118.5</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -22980,7 +23062,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -23006,7 +23088,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -23096,7 +23178,7 @@
         <v>310</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -23186,13 +23268,13 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -23339,24 +23421,24 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{245A1644-2BFB-4EA7-BEAA-4598893697AD}">
   <dimension ref="A1:AJ29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -23367,7 +23449,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -23379,7 +23461,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -23390,7 +23472,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -23513,7 +23595,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -23578,7 +23660,7 @@
         <v>48.012999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -23643,7 +23725,7 @@
         <v>11.5</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -23711,13 +23793,13 @@
         <v>95.1</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -23797,7 +23879,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -23823,7 +23905,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -23928,7 +24010,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -23994,13 +24076,13 @@
         <v>44</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -24137,12 +24219,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
       <c r="L16" t="s">
         <v>19</v>
       </c>
     </row>
-    <row r="29" spans="18:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="18:18" x14ac:dyDescent="0.3">
       <c r="R29">
         <f>485*1.03</f>
         <v>499.55</v>
@@ -24158,24 +24240,24 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB28D160-17A5-469E-8CF6-067E3CB95279}">
   <dimension ref="A1:AJ29"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -24186,7 +24268,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -24195,7 +24277,7 @@
         <v>379.31</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -24203,7 +24285,7 @@
         <v>384</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -24326,7 +24408,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -24361,7 +24443,7 @@
         <v>2.0994000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -24396,7 +24478,7 @@
         <v>-105</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -24434,13 +24516,13 @@
         <v>76.599999999999994</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -24500,7 +24582,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -24526,7 +24608,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -24631,7 +24713,7 @@
         <v>275</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -24667,13 +24749,13 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -24810,13 +24892,13 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="10:18" x14ac:dyDescent="0.35">
+    <row r="18" spans="10:18" x14ac:dyDescent="0.3">
       <c r="J18">
         <f>1-348/457</f>
         <v>0.23851203501094087</v>
       </c>
     </row>
-    <row r="29" spans="10:18" x14ac:dyDescent="0.35">
+    <row r="29" spans="10:18" x14ac:dyDescent="0.3">
       <c r="R29">
         <f>485*1.03</f>
         <v>499.55</v>
@@ -24832,22 +24914,22 @@
 <file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{026B26E4-CFF3-41E2-8721-B0918FFC9B0E}">
   <dimension ref="A1:AK36"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="2" max="2" width="39.81640625" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="19.453125" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.77734375" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="19.44140625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="18.5546875" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="18.109375" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="17.21875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>79</v>
       </c>
       <c r="B1" s="3"/>
     </row>
-    <row r="2" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>71</v>
       </c>
@@ -24859,7 +24941,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>70</v>
       </c>
@@ -24876,7 +24958,7 @@
         <v>0.13778705636743216</v>
       </c>
     </row>
-    <row r="4" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -24885,28 +24967,11 @@
         <v>0</v>
       </c>
       <c r="E4" t="s">
-        <v>59</v>
-      </c>
-      <c r="M4" t="s">
-        <v>73</v>
-      </c>
-      <c r="N4" t="s">
-        <v>74</v>
-      </c>
-      <c r="O4" s="3" t="s">
-        <v>75</v>
-      </c>
-      <c r="P4" t="s">
-        <v>76</v>
-      </c>
-      <c r="Q4" t="s">
-        <v>77</v>
-      </c>
-      <c r="R4" t="s">
-        <v>78</v>
-      </c>
-    </row>
-    <row r="5" spans="1:37" x14ac:dyDescent="0.35">
+        <v>60</v>
+      </c>
+      <c r="O4" s="3"/>
+    </row>
+    <row r="5" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A5" s="10"/>
       <c r="B5" s="4" t="s">
         <v>0</v>
@@ -25005,7 +25070,7 @@
       <c r="AJ5" s="10"/>
       <c r="AK5" s="10"/>
     </row>
-    <row r="6" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A6" s="3"/>
       <c r="B6" s="5" t="s">
         <v>1</v>
@@ -25034,8 +25099,38 @@
       <c r="J6">
         <v>65.655000000000001</v>
       </c>
-    </row>
-    <row r="7" spans="1:37" x14ac:dyDescent="0.35">
+      <c r="K6">
+        <v>63.7</v>
+      </c>
+      <c r="L6">
+        <v>61.6</v>
+      </c>
+      <c r="M6">
+        <v>60.4</v>
+      </c>
+      <c r="N6">
+        <v>2.2599999999999998</v>
+      </c>
+      <c r="O6">
+        <v>9.8000000000000007</v>
+      </c>
+      <c r="P6">
+        <v>21</v>
+      </c>
+      <c r="Q6">
+        <v>44</v>
+      </c>
+      <c r="R6">
+        <v>55.9</v>
+      </c>
+      <c r="S6">
+        <v>67.599999999999994</v>
+      </c>
+      <c r="T6">
+        <v>75.8</v>
+      </c>
+    </row>
+    <row r="7" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A7" s="3"/>
       <c r="B7" s="6" t="s">
         <v>2</v>
@@ -25064,8 +25159,38 @@
       <c r="J7">
         <v>-24.202999999999999</v>
       </c>
-    </row>
-    <row r="8" spans="1:37" x14ac:dyDescent="0.35">
+      <c r="K7">
+        <v>-25.6</v>
+      </c>
+      <c r="L7">
+        <v>-16</v>
+      </c>
+      <c r="M7">
+        <v>-20.6</v>
+      </c>
+      <c r="N7">
+        <v>-70.81</v>
+      </c>
+      <c r="O7">
+        <v>-63</v>
+      </c>
+      <c r="P7">
+        <v>-53.6</v>
+      </c>
+      <c r="Q7">
+        <v>-39.280999999999999</v>
+      </c>
+      <c r="R7">
+        <v>-29.6</v>
+      </c>
+      <c r="S7">
+        <v>-16.3</v>
+      </c>
+      <c r="T7">
+        <v>-10.199999999999999</v>
+      </c>
+    </row>
+    <row r="8" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A8" s="3"/>
       <c r="B8" s="4" t="s">
         <v>47</v>
@@ -25094,8 +25219,38 @@
       <c r="J8">
         <v>622.85</v>
       </c>
-    </row>
-    <row r="9" spans="1:37" x14ac:dyDescent="0.35">
+      <c r="K8">
+        <v>622.79999999999995</v>
+      </c>
+      <c r="L8">
+        <v>623.6</v>
+      </c>
+      <c r="M8">
+        <v>622</v>
+      </c>
+      <c r="N8">
+        <v>626</v>
+      </c>
+      <c r="O8">
+        <v>624</v>
+      </c>
+      <c r="P8">
+        <v>622</v>
+      </c>
+      <c r="Q8">
+        <v>625.1</v>
+      </c>
+      <c r="R8">
+        <v>625.1</v>
+      </c>
+      <c r="S8">
+        <v>623.6</v>
+      </c>
+      <c r="T8">
+        <v>623</v>
+      </c>
+    </row>
+    <row r="9" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -25126,16 +25281,36 @@
       <c r="J9" s="1">
         <v>83</v>
       </c>
-      <c r="K9" s="1"/>
-      <c r="L9" s="1"/>
-      <c r="M9" s="1"/>
-      <c r="N9" s="1"/>
-      <c r="O9" s="1"/>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="1"/>
+      <c r="K9" s="1">
+        <v>57.5</v>
+      </c>
+      <c r="L9" s="1">
+        <v>88</v>
+      </c>
+      <c r="M9" s="1">
+        <v>89</v>
+      </c>
+      <c r="N9" s="1">
+        <v>84.5</v>
+      </c>
+      <c r="O9" s="1">
+        <v>87.5</v>
+      </c>
+      <c r="P9" s="1">
+        <v>87</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>89</v>
+      </c>
+      <c r="R9" s="1">
+        <v>90</v>
+      </c>
+      <c r="S9" s="1">
+        <v>88.5</v>
+      </c>
+      <c r="T9" s="1">
+        <v>26.5</v>
+      </c>
       <c r="U9" s="1"/>
       <c r="V9" s="1"/>
       <c r="W9" s="1"/>
@@ -25154,7 +25329,7 @@
       <c r="AJ9" s="1"/>
       <c r="AK9" s="1"/>
     </row>
-    <row r="10" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -25162,42 +25337,59 @@
       <c r="C10" s="16">
         <v>408</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10">
         <v>410</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10">
         <v>421</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10">
         <v>427</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10">
         <v>437</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10">
         <v>441</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10">
         <v>444</v>
       </c>
-      <c r="J10" s="33">
+      <c r="J10">
         <v>447</v>
       </c>
-      <c r="K10" s="33"/>
-      <c r="L10" s="33"/>
-      <c r="M10" s="33"/>
-      <c r="N10" s="33"/>
-      <c r="O10" s="33"/>
-      <c r="P10" s="33"/>
-      <c r="Q10" s="33"/>
-      <c r="R10" s="33"/>
-      <c r="S10" s="33"/>
-      <c r="T10" s="33"/>
-      <c r="U10" s="33"/>
-      <c r="V10" s="33"/>
-      <c r="W10" s="33"/>
-    </row>
-    <row r="11" spans="1:37" x14ac:dyDescent="0.35">
+      <c r="K10" s="33">
+        <v>445</v>
+      </c>
+      <c r="L10" s="33">
+        <v>452</v>
+      </c>
+      <c r="M10" s="33">
+        <v>449</v>
+      </c>
+      <c r="N10" s="33">
+        <v>403</v>
+      </c>
+      <c r="O10" s="33">
+        <v>407</v>
+      </c>
+      <c r="P10" s="33">
+        <v>415</v>
+      </c>
+      <c r="Q10" s="33">
+        <v>430</v>
+      </c>
+      <c r="R10" s="33">
+        <v>438</v>
+      </c>
+      <c r="S10" s="33">
+        <v>450</v>
+      </c>
+      <c r="T10" s="33">
+        <v>453</v>
+      </c>
+    </row>
+    <row r="11" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -25240,44 +25432,44 @@
       <c r="AJ11" s="1"/>
       <c r="AK11" s="1"/>
     </row>
-    <row r="12" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="16"/>
     </row>
-    <row r="13" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
       </c>
       <c r="C13" s="16">
-        <v>249.71</v>
-      </c>
-      <c r="D13">
-        <v>249.71</v>
-      </c>
-      <c r="E13">
-        <v>249.71</v>
-      </c>
-      <c r="F13">
-        <v>249.71</v>
-      </c>
-      <c r="G13">
-        <v>249.71</v>
-      </c>
-      <c r="H13">
-        <v>249.71</v>
-      </c>
-      <c r="I13">
-        <v>249.71</v>
-      </c>
-      <c r="J13">
-        <v>249.71</v>
-      </c>
-      <c r="K13">
-        <v>249.71</v>
+        <v>260.20999999999998</v>
+      </c>
+      <c r="D13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="E13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="F13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="G13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="H13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="I13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="J13" s="16">
+        <v>260.20999999999998</v>
+      </c>
+      <c r="K13" s="16">
+        <v>260.20999999999998</v>
       </c>
       <c r="L13">
         <v>249.71</v>
@@ -25340,7 +25532,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -25369,8 +25561,38 @@
       <c r="J14">
         <v>77</v>
       </c>
-    </row>
-    <row r="15" spans="1:37" x14ac:dyDescent="0.35">
+      <c r="K14">
+        <v>75</v>
+      </c>
+      <c r="L14">
+        <v>74</v>
+      </c>
+      <c r="M14">
+        <v>75</v>
+      </c>
+      <c r="N14">
+        <v>55</v>
+      </c>
+      <c r="O14">
+        <v>65</v>
+      </c>
+      <c r="P14">
+        <v>75</v>
+      </c>
+      <c r="Q14">
+        <v>76</v>
+      </c>
+      <c r="R14">
+        <v>75</v>
+      </c>
+      <c r="S14">
+        <v>75</v>
+      </c>
+      <c r="T14">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="15" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
@@ -25392,7 +25614,9 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
-      <c r="T15" s="2"/>
+      <c r="T15" s="2" t="s">
+        <v>81</v>
+      </c>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
@@ -25411,213 +25635,213 @@
       <c r="AJ15" s="2"/>
       <c r="AK15" s="2"/>
     </row>
-    <row r="16" spans="1:37" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A16" s="3"/>
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
       <c r="C16" s="16">
-        <f>-C6*SIN(RADIANS(C9+5.15))*C13/1000</f>
-        <v>-1.9089163300292105</v>
+        <f>-C6*SIN(RADIANS(C9+4.96))*C13/1000</f>
+        <v>-1.9888446022622024</v>
       </c>
       <c r="D16" s="16">
-        <f t="shared" ref="D16:AE16" si="0">-D6*SIN(RADIANS(D9+5.15))*D13/1000</f>
-        <v>-4.0809375058192954</v>
+        <f t="shared" ref="D16:K16" si="0">-D6*SIN(RADIANS(D9+4.96))*D13/1000</f>
+        <v>-4.2527956349925518</v>
       </c>
       <c r="E16" s="16">
         <f t="shared" si="0"/>
-        <v>-7.0574220518637798</v>
+        <v>-7.3539886035989408</v>
       </c>
       <c r="F16" s="16">
         <f t="shared" si="0"/>
-        <v>-10.09453321766197</v>
+        <v>-10.527409285407064</v>
       </c>
       <c r="G16" s="16">
         <f t="shared" si="0"/>
-        <v>-13.401234911810583</v>
+        <v>-13.966402193997661</v>
       </c>
       <c r="H16" s="16">
         <f t="shared" si="0"/>
-        <v>-14.847761858930939</v>
+        <v>-15.473036951197667</v>
       </c>
       <c r="I16" s="16">
         <f t="shared" si="0"/>
-        <v>-15.781617917093591</v>
+        <v>-16.445267992387105</v>
       </c>
       <c r="J16" s="16">
         <f t="shared" si="0"/>
-        <v>-16.386164614410578</v>
+        <v>-17.07325998043143</v>
       </c>
       <c r="K16" s="16">
         <f t="shared" si="0"/>
+        <v>-14.697192119709124</v>
+      </c>
+      <c r="L16" s="16">
+        <f t="shared" ref="D16:AE16" si="1">-L6*SIN(RADIANS(L9+5.15))*L13/1000</f>
+        <v>-15.358895091501429</v>
+      </c>
+      <c r="M16" s="16">
+        <f t="shared" si="1"/>
+        <v>-15.042937875530633</v>
+      </c>
+      <c r="N16" s="16">
+        <f t="shared" si="1"/>
+        <v>-0.56433407059449248</v>
+      </c>
+      <c r="O16" s="16">
+        <f t="shared" si="1"/>
+        <v>-2.4445410159422072</v>
+      </c>
+      <c r="P16" s="16">
+        <f t="shared" si="1"/>
+        <v>-5.2402184740344895</v>
+      </c>
+      <c r="Q16" s="16">
+        <f t="shared" si="1"/>
+        <v>-10.95843156495609</v>
+      </c>
+      <c r="R16" s="16">
+        <f t="shared" si="1"/>
+        <v>-13.902438921694182</v>
+      </c>
+      <c r="S16" s="16">
+        <f t="shared" si="1"/>
+        <v>-16.846155017276384</v>
+      </c>
+      <c r="T16" s="16">
+        <f t="shared" si="1"/>
+        <v>-9.9320795468220986</v>
+      </c>
+      <c r="U16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="L16" s="16">
-        <f t="shared" si="0"/>
+      <c r="V16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="M16" s="16">
-        <f t="shared" si="0"/>
+      <c r="W16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="N16" s="16">
-        <f t="shared" si="0"/>
+      <c r="X16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="O16" s="16">
-        <f t="shared" si="0"/>
+      <c r="Y16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="P16" s="16">
-        <f t="shared" si="0"/>
+      <c r="Z16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="Q16" s="16">
-        <f t="shared" si="0"/>
+      <c r="AA16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="R16" s="16">
-        <f t="shared" si="0"/>
+      <c r="AB16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="S16" s="16">
-        <f t="shared" si="0"/>
+      <c r="AC16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="T16" s="16">
-        <f t="shared" si="0"/>
+      <c r="AD16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="U16" s="16">
-        <f t="shared" si="0"/>
+      <c r="AE16" s="16">
+        <f t="shared" si="1"/>
         <v>0</v>
       </c>
-      <c r="V16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="W16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Y16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AB16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AC16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AD16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AE16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
     </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A18" s="3"/>
       <c r="B18" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A27" s="3"/>
       <c r="B27" s="29" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A33" s="3"/>
       <c r="B33" s="3"/>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A34" s="3"/>
       <c r="B34" s="3"/>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A35" s="3"/>
       <c r="B35" s="3"/>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.3">
       <c r="A36" s="3"/>
       <c r="B36" s="3"/>
     </row>
@@ -25631,24 +25855,24 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26D1208C-7CDD-421F-9FF0-096EE144B4F3}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -25659,7 +25883,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -25668,7 +25892,7 @@
         <v>379.31</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -25680,7 +25904,7 @@
         <v>0.16849015317286653</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -25803,7 +26027,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -25895,7 +26119,7 @@
         <v>24.667000000000002</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -25987,7 +26211,7 @@
         <v>-123</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -26082,13 +26306,13 @@
         <v>81.400000000000006</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -26186,7 +26410,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -26212,7 +26436,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -26317,7 +26541,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -26410,13 +26634,13 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -26563,24 +26787,24 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{23CB8201-A5D3-4826-B613-98BAA3DB341B}">
   <dimension ref="A1:AJ15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -26591,7 +26815,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -26600,7 +26824,7 @@
         <v>403.38</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -26612,7 +26836,7 @@
         <v>0.18106995884773658</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -26735,7 +26959,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -26752,7 +26976,7 @@
         <v>13.111000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -26769,7 +26993,7 @@
         <v>-92</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -26789,13 +27013,13 @@
         <v>80.7</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -26843,7 +27067,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -26869,7 +27093,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -26974,7 +27198,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -26992,13 +27216,13 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -27145,24 +27369,24 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D539E524-5F19-4B4B-B21A-C95F2596B6A0}">
   <dimension ref="A1:AJ27"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>29</v>
       </c>
     </row>
-    <row r="2" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -27173,7 +27397,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B3" s="3" t="s">
         <v>14</v>
       </c>
@@ -27185,7 +27409,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="4" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B4" s="3" t="s">
         <v>17</v>
       </c>
@@ -27206,7 +27430,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:36" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -27329,7 +27553,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="6" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -27415,7 +27639,7 @@
         <v>33.061999999999998</v>
       </c>
     </row>
-    <row r="7" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -27498,7 +27722,7 @@
         <v>-66</v>
       </c>
     </row>
-    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -27584,13 +27808,13 @@
         <v>83.5</v>
       </c>
     </row>
-    <row r="9" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:36" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -27682,7 +27906,7 @@
       <c r="AI10" s="2"/>
       <c r="AJ10" s="2"/>
     </row>
-    <row r="11" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -27708,7 +27932,7 @@
       <c r="S11" s="1"/>
       <c r="T11" s="1"/>
     </row>
-    <row r="12" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -27813,7 +28037,7 @@
         <v>267</v>
       </c>
     </row>
-    <row r="13" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:36" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -27897,13 +28121,13 @@
         <v>28</v>
       </c>
     </row>
-    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:36" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:36" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -28040,7 +28264,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:36" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:36" x14ac:dyDescent="0.3">
       <c r="U16" t="s">
         <v>23</v>
       </c>
@@ -28048,22 +28272,22 @@
         <v>25</v>
       </c>
     </row>
-    <row r="17" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="17" spans="17:29" x14ac:dyDescent="0.3">
       <c r="AB17">
         <v>2.2241</v>
       </c>
     </row>
-    <row r="18" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="18" spans="17:29" x14ac:dyDescent="0.3">
       <c r="AC18" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="24" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="24" spans="17:29" x14ac:dyDescent="0.3">
       <c r="Q24" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="25" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="25" spans="17:29" x14ac:dyDescent="0.3">
       <c r="Q25" t="s">
         <v>42</v>
       </c>
@@ -28074,7 +28298,7 @@
         <v>-1.4999999999999999E-2</v>
       </c>
     </row>
-    <row r="26" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="26" spans="17:29" x14ac:dyDescent="0.3">
       <c r="Q26" t="s">
         <v>43</v>
       </c>
@@ -28085,7 +28309,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="27" spans="17:29" x14ac:dyDescent="0.35">
+    <row r="27" spans="17:29" x14ac:dyDescent="0.3">
       <c r="R27">
         <v>505</v>
       </c>
@@ -28100,24 +28324,24 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{66E6C766-4925-4D35-B304-44784D2D9843}">
   <dimension ref="A1:Q16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>38</v>
       </c>
     </row>
-    <row r="2" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -28128,7 +28352,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -28136,7 +28360,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="4" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -28147,7 +28371,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:17" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -28197,7 +28421,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="6" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -28244,7 +28468,7 @@
         <v>6.2092000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -28291,7 +28515,7 @@
         <v>-18.5</v>
       </c>
     </row>
-    <row r="8" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -28341,7 +28565,7 @@
         <v>90.5</v>
       </c>
     </row>
-    <row r="9" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>3</v>
@@ -28389,7 +28613,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="10" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>8</v>
       </c>
@@ -28397,13 +28621,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -28454,7 +28678,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="13" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -28502,13 +28726,13 @@
         <v>24</v>
       </c>
     </row>
-    <row r="14" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:17" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:17" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -28573,7 +28797,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:17" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:17" x14ac:dyDescent="0.3">
       <c r="L16" t="s">
         <v>39</v>
       </c>
@@ -28588,24 +28812,24 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B944D1C8-56B8-47D8-90D4-245D22EBCA01}">
   <dimension ref="A1:AE15"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="9.08984375" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="9.109375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>66</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -28616,7 +28840,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -28624,7 +28848,7 @@
         <v>350</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -28632,7 +28856,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -28724,7 +28948,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -28780,7 +29004,7 @@
         <v>17.72</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -28836,7 +29060,7 @@
         <v>-119.5</v>
       </c>
     </row>
-    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A8" s="11" t="s">
         <v>7</v>
       </c>
@@ -28895,7 +29119,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="9" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A9" s="12"/>
       <c r="B9" s="8" t="s">
         <v>3</v>
@@ -28952,7 +29176,7 @@
         <v>395</v>
       </c>
     </row>
-    <row r="10" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A10" s="11" t="s">
         <v>8</v>
       </c>
@@ -28960,13 +29184,13 @@
         <v>9</v>
       </c>
     </row>
-    <row r="11" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A11" s="12"/>
       <c r="B11" s="8" t="s">
         <v>33</v>
       </c>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>10</v>
@@ -29059,7 +29283,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>11</v>
@@ -29116,13 +29340,13 @@
         <v>36</v>
       </c>
     </row>
-    <row r="14" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A14" s="13"/>
       <c r="B14" s="9" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="15" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B15" s="5" t="s">
         <v>6</v>
       </c>
@@ -29253,25 +29477,25 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{07511B1B-CFA9-4E3E-A27D-F86FFAE12463}">
   <dimension ref="A1:AE16"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="8" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>65</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -29282,7 +29506,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -29290,7 +29514,7 @@
         <v>345</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -29301,7 +29525,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -29393,7 +29617,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -29416,7 +29640,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -29436,7 +29660,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B8" s="7" t="s">
         <v>47</v>
       </c>
@@ -29456,7 +29680,7 @@
         <v>628.9</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -29479,7 +29703,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -29501,7 +29725,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -29510,14 +29734,14 @@
       </c>
       <c r="C11" s="24"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="8" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="23"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -29589,7 +29813,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -29608,14 +29832,14 @@
         <v>57</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="9" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="25"/>
     </row>
-    <row r="16" spans="1:31" s="28" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" s="28" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A16" s="26"/>
       <c r="B16" s="27" t="s">
         <v>6</v>
@@ -29735,26 +29959,26 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{CC7A6C4B-FDDD-4D0B-90C8-5B01A1705645}">
   <dimension ref="A1:AE17"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.81640625" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="8" width="19.6328125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.77734375" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="19.6640625" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="14" max="14" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>64</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -29765,7 +29989,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -29773,7 +29997,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -29790,7 +30014,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -29882,7 +30106,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -29926,7 +30150,7 @@
         <v>37.6</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -29970,7 +30194,7 @@
         <v>-73</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B8" s="7" t="s">
         <v>47</v>
       </c>
@@ -30014,7 +30238,7 @@
         <v>629.71799999999996</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -30061,7 +30285,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -30106,7 +30330,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -30115,14 +30339,14 @@
       </c>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="16"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -30194,7 +30418,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -30239,14 +30463,14 @@
         <v>26</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="14"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
@@ -30367,7 +30591,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="14:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="14:15" x14ac:dyDescent="0.3">
       <c r="N17" s="3" t="s">
         <v>50</v>
       </c>
@@ -30385,27 +30609,27 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{AB4D735A-7F76-4974-8609-056275EBAB78}">
   <dimension ref="A1:AE21"/>
-  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="8.90625" style="3"/>
-    <col min="2" max="2" width="19.6328125" style="3" customWidth="1"/>
-    <col min="3" max="3" width="12.36328125" customWidth="1"/>
-    <col min="5" max="5" width="8.6328125" customWidth="1"/>
-    <col min="6" max="6" width="11.36328125" customWidth="1"/>
-    <col min="7" max="7" width="13.36328125" customWidth="1"/>
-    <col min="8" max="8" width="12.453125" customWidth="1"/>
-    <col min="9" max="9" width="13.453125" customWidth="1"/>
+    <col min="1" max="1" width="8.88671875" style="3"/>
+    <col min="2" max="2" width="19.6640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="12.33203125" customWidth="1"/>
+    <col min="5" max="5" width="8.6640625" customWidth="1"/>
+    <col min="6" max="6" width="11.33203125" customWidth="1"/>
+    <col min="7" max="7" width="13.33203125" customWidth="1"/>
+    <col min="8" max="8" width="12.44140625" customWidth="1"/>
+    <col min="9" max="9" width="13.44140625" customWidth="1"/>
     <col min="10" max="10" width="14" customWidth="1"/>
-    <col min="12" max="12" width="12.90625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="14.90625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="12.88671875" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
         <v>63</v>
       </c>
     </row>
-    <row r="2" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>5</v>
       </c>
@@ -30416,7 +30640,7 @@
         <v>46</v>
       </c>
     </row>
-    <row r="3" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A3" s="3" t="s">
         <v>36</v>
       </c>
@@ -30432,7 +30656,7 @@
         <v>0.14749999999999996</v>
       </c>
     </row>
-    <row r="4" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A4" s="3" t="s">
         <v>35</v>
       </c>
@@ -30450,7 +30674,7 @@
       </c>
       <c r="O4" s="3"/>
     </row>
-    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:31" s="10" customFormat="1" x14ac:dyDescent="0.3">
       <c r="B5" s="4" t="s">
         <v>0</v>
       </c>
@@ -30542,7 +30766,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="6" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B6" s="5" t="s">
         <v>1</v>
       </c>
@@ -30580,7 +30804,7 @@
         <v>45.42</v>
       </c>
     </row>
-    <row r="7" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B7" s="6" t="s">
         <v>2</v>
       </c>
@@ -30618,7 +30842,7 @@
         <v>-52.89</v>
       </c>
     </row>
-    <row r="8" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B8" s="4" t="s">
         <v>47</v>
       </c>
@@ -30656,7 +30880,7 @@
         <v>623.61</v>
       </c>
     </row>
-    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A9" s="11" t="s">
         <v>7</v>
       </c>
@@ -30703,7 +30927,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="10" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A10" s="12"/>
       <c r="B10" s="8" t="s">
         <v>3</v>
@@ -30748,7 +30972,7 @@
         <v>396</v>
       </c>
     </row>
-    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:31" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A11" s="11" t="s">
         <v>8</v>
       </c>
@@ -30757,14 +30981,14 @@
       </c>
       <c r="C11" s="15"/>
     </row>
-    <row r="12" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A12" s="12"/>
       <c r="B12" s="18" t="s">
         <v>33</v>
       </c>
       <c r="C12" s="16"/>
     </row>
-    <row r="13" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A13" s="12"/>
       <c r="B13" s="8" t="s">
         <v>10</v>
@@ -30857,7 +31081,7 @@
         <v>249.71</v>
       </c>
     </row>
-    <row r="14" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:31" x14ac:dyDescent="0.3">
       <c r="A14" s="12"/>
       <c r="B14" s="8" t="s">
         <v>11</v>
@@ -30896,14 +31120,14 @@
         <v>27</v>
       </c>
     </row>
-    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:31" s="2" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A15" s="13"/>
       <c r="B15" s="19" t="s">
         <v>4</v>
       </c>
       <c r="C15" s="14"/>
     </row>
-    <row r="16" spans="1:31" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:31" x14ac:dyDescent="0.3">
       <c r="B16" s="5" t="s">
         <v>6</v>
       </c>
@@ -31024,11 +31248,11 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="17" spans="2:15" x14ac:dyDescent="0.3">
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
     </row>
-    <row r="21" spans="2:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="2:15" x14ac:dyDescent="0.3">
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>

</xml_diff>

<commit_message>
Knee Flexor Optimizer updated
to find Xi0 - Xi2
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9920989-4A16-4DCE-8028-31F803D33A95}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C89EFDFE-5E7B-4363-A0D8-5ADE892DBC2B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" firstSheet="7" activeTab="8" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="11" activeTab="16" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest10mm_1" sheetId="9" r:id="rId1"/>
@@ -31,10 +31,21 @@
     <sheet name="FlxTest10mm_4" sheetId="23" r:id="rId16"/>
     <sheet name="FlxTest10mm_5" sheetId="24" r:id="rId17"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
+    </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
     </ext>
   </extLst>
 </workbook>
@@ -49,36 +60,18 @@
   <commentList>
     <comment ref="D3" authorId="0" shapeId="0" xr:uid="{31540696-8989-4ECF-9DA4-105271D5E559}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="1" shapeId="0" xr:uid="{4ABBB369-E711-4E3D-9229-46727333D172}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -97,87 +90,42 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{29300245-EF40-4E4F-8F6D-1266C425EACE}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{00298076-0747-4A6C-9F96-1B56DD480064}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{BDF31CF8-F642-45F3-81CA-9C8FF04449E8}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="3" shapeId="0" xr:uid="{C8A435E7-474C-41D6-A569-7731B05DEC1C}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
     <comment ref="C4" authorId="4" shapeId="0" xr:uid="{6E231C95-A9F8-4BE0-A13C-7D1696721C9B}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     So it can reach -114 degrees</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -196,87 +144,42 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{7429FFDB-7320-40ED-9095-CADFEE0453D3}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{56BB9B1E-AE6F-4367-98DA-1738BC17BA33}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{181A90AF-6CB1-444A-AC50-05218AF784A8}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="3" shapeId="0" xr:uid="{E9CB4941-5049-48DD-9386-0FE986486E00}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
     <comment ref="C4" authorId="4" shapeId="0" xr:uid="{4B24DE55-490A-4648-B1F6-ECBEA4FEDB7F}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     So it can reach -114 degrees</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -295,87 +198,42 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{F99A6D76-844F-423C-8E72-632020492202}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{57404540-41ED-4CFC-A34A-B0C06D36E435}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{FD23BCFD-5D0D-499D-B1BC-4D31A4174384}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="3" shapeId="0" xr:uid="{34C2BEB3-8987-42FD-9240-D19AB0F3395E}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
     <comment ref="C4" authorId="4" shapeId="0" xr:uid="{619279C5-5896-4658-A891-94E7656E0604}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     So it can reach -114 degrees</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -394,87 +252,42 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{B3DD3E36-DE23-4526-822F-7544076C12AF}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{44F69930-AA26-4737-9556-6F232E8AC193}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{6E9C7D1B-6D13-4A15-A63C-B49E3DDDDD72}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="3" shapeId="0" xr:uid="{A117DFD4-25AF-41A6-9D26-99F7C9197E59}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
     <comment ref="C4" authorId="4" shapeId="0" xr:uid="{70F2E1CB-BEA3-46AD-8012-48E9D04ADA3E}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     So it can reach -114 degrees</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -493,87 +306,42 @@
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{1412A674-61A3-4D66-9D3E-5374366576D7}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="C3" authorId="1" shapeId="0" xr:uid="{7BAEFA08-D790-466D-A190-320CBA26570E}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Recheck after test</t>
-        </r>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{E1852E19-B84C-463E-A0CB-BF0ADA1DC1BE}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Max contracted length normalized by resting length</t>
-        </r>
       </text>
     </comment>
     <comment ref="E3" authorId="3" shapeId="0" xr:uid="{13B25287-2F50-4E04-AC48-02AB262B1DE9}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-        </r>
       </text>
     </comment>
     <comment ref="C4" authorId="4" shapeId="0" xr:uid="{50243B4E-1A69-4602-BC70-D861CF3BE17E}">
       <text>
-        <r>
-          <rPr>
-            <sz val="11"/>
-            <color theme="1"/>
-            <rFont val="Calibri"/>
-            <family val="2"/>
-            <scheme val="minor"/>
-          </rPr>
-          <t>[Threaded comment]
+        <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Initially measured 30 mm but noticed it was actually 35 mm around data reading 6</t>
-        </r>
       </text>
     </comment>
   </commentList>
@@ -581,7 +349,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="394" uniqueCount="99">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="395" uniqueCount="98">
   <si>
     <t>Test #</t>
   </si>
@@ -824,9 +592,6 @@
   </si>
   <si>
     <t>^Collected by Moe &amp; Ben</t>
-  </si>
-  <si>
-    <t>oooooo</t>
   </si>
   <si>
     <t>Flex test 5</t>
@@ -19808,16 +19573,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>11</xdr:col>
-      <xdr:colOff>410920</xdr:colOff>
+      <xdr:col>3</xdr:col>
+      <xdr:colOff>572285</xdr:colOff>
       <xdr:row>21</xdr:row>
-      <xdr:rowOff>46935</xdr:rowOff>
+      <xdr:rowOff>73829</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>1130338</xdr:colOff>
+      <xdr:col>11</xdr:col>
+      <xdr:colOff>242832</xdr:colOff>
       <xdr:row>36</xdr:row>
-      <xdr:rowOff>78684</xdr:rowOff>
+      <xdr:rowOff>105578</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -20194,9 +19959,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -20234,7 +19999,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -20340,7 +20105,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -20482,7 +20247,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -22239,7 +22004,7 @@
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
       <c r="N22" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="23" spans="2:15" x14ac:dyDescent="0.3">
@@ -22943,7 +22708,7 @@
         <v>52</v>
       </c>
       <c r="O21" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">
@@ -23887,7 +23652,7 @@
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
       <c r="O24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25" spans="1:15" x14ac:dyDescent="0.3">
@@ -26380,15 +26145,15 @@
       </c>
       <c r="B3" s="3"/>
       <c r="C3">
-        <v>413</v>
+        <v>403</v>
       </c>
       <c r="D3">
         <f>(C3/C2)</f>
-        <v>0.86221294363256784</v>
+        <v>0.84133611691022969</v>
       </c>
       <c r="E3">
         <f>1-D3</f>
-        <v>0.13778705636743216</v>
+        <v>0.15866388308977031</v>
       </c>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.3">
@@ -27047,9 +26812,7 @@
       <c r="Q15" s="2"/>
       <c r="R15" s="2"/>
       <c r="S15" s="2"/>
-      <c r="T15" s="2" t="s">
-        <v>81</v>
-      </c>
+      <c r="T15" s="2"/>
       <c r="U15" s="2"/>
       <c r="V15" s="2"/>
       <c r="W15" s="2"/>
@@ -27209,12 +26972,19 @@
     <row r="20" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
+      <c r="M20" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="21" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A21" s="3"/>
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
+      <c r="M21">
+        <f>AVERAGE(C8:T8)</f>
+        <v>623.16511111111129</v>
+      </c>
     </row>
     <row r="22" spans="1:15" x14ac:dyDescent="0.3">
       <c r="A22" s="3"/>
@@ -27280,8 +27050,9 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-  <legacyDrawing r:id="rId2"/>
+  <pageSetup orientation="portrait" horizontalDpi="0" verticalDpi="0" r:id="rId1"/>
+  <drawing r:id="rId2"/>
+  <legacyDrawing r:id="rId3"/>
 </worksheet>
 </file>
 
@@ -27301,7 +27072,7 @@
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.3">
       <c r="A1" s="3" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B1" s="3"/>
     </row>
@@ -27346,14 +27117,14 @@
         <v>59</v>
       </c>
       <c r="H4" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="O4" s="3"/>
       <c r="Q4" t="s">
         <v>26</v>
       </c>
       <c r="R4" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="5" spans="1:37" x14ac:dyDescent="0.3">
@@ -28161,24 +27932,24 @@
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="H17" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
       <c r="Q17" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="R17" t="s">
+        <v>87</v>
+      </c>
+      <c r="S17" t="s">
         <v>88</v>
       </c>
-      <c r="S17" t="s">
-        <v>89</v>
-      </c>
       <c r="T17" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="U17" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="18" spans="1:21" x14ac:dyDescent="0.3">
@@ -28187,13 +27958,13 @@
         <v>72</v>
       </c>
       <c r="H18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="S18" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="T18" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.3">
@@ -28221,10 +27992,17 @@
     <row r="24" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
+      <c r="M24" t="s">
+        <v>93</v>
+      </c>
     </row>
     <row r="25" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
+      <c r="M25">
+        <f>AVERAGE(C8:U8)</f>
+        <v>623.42526315789462</v>
+      </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.3">
       <c r="A26" s="3"/>
@@ -32376,7 +32154,7 @@
     </row>
     <row r="18" spans="8:8" x14ac:dyDescent="0.3">
       <c r="H18" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
     </row>
   </sheetData>
@@ -33031,7 +32809,7 @@
     </row>
     <row r="19" spans="14:15" x14ac:dyDescent="0.3">
       <c r="O19" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -33692,7 +33470,7 @@
         <v>52</v>
       </c>
       <c r="N21" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="22" spans="2:15" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
Finished collecting data for EXT 465mm Muscle
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\melze\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7C53A715-A518-499E-84CF-594F33F4204D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4A3E813-9C1F-4DCB-941F-46896A883EB7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="41085" yWindow="-16200" windowWidth="14610" windowHeight="15585" firstSheet="11" activeTab="12" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
   </bookViews>
@@ -349,7 +349,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="377" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="87">
   <si>
     <t>Test #</t>
   </si>
@@ -604,6 +604,12 @@
   </si>
   <si>
     <t>Ext Test 12</t>
+  </si>
+  <si>
+    <t>* Pretensioned to 0.935 N</t>
+  </si>
+  <si>
+    <t>* Pretensioned to 0.975 N</t>
   </si>
 </sst>
 </file>
@@ -3098,10 +3104,10 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>ExtTest10mm_13!$C$7:$S$7</c:f>
+              <c:f>ExtTest10mm_13!$C$7:$AE$7</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="17"/>
+                <c:ptCount val="29"/>
                 <c:pt idx="0">
                   <c:v>23.184999999999999</c:v>
                 </c:pt>
@@ -3140,6 +3146,45 @@
                 </c:pt>
                 <c:pt idx="12">
                   <c:v>-55.795000000000002</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>-60.820999999999998</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>-67.641999999999996</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>-73.385999999999996</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>-84.156000000000006</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>-90.259</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>-75.180999999999997</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>-65.846999999999994</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>-51.487000000000002</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>-33.896000000000001</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>-17.023</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>-4.0990000000000002</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>6.3120000000000003</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>16.004999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -3190,43 +3235,43 @@
                   <c:v>3.8508462486362252</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0</c:v>
+                  <c:v>3.6291506505175044</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0</c:v>
+                  <c:v>4.1829161707816302</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0</c:v>
+                  <c:v>4.4642414453654187</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0</c:v>
+                  <c:v>5.3517587170964296</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0</c:v>
+                  <c:v>5.5243356546689117</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>0</c:v>
+                  <c:v>4.6434882022501975</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>0</c:v>
+                  <c:v>3.9337462112650874</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>0</c:v>
+                  <c:v>3.2362035092330919</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>0</c:v>
+                  <c:v>2.4284517189520791</c:v>
                 </c:pt>
                 <c:pt idx="22">
-                  <c:v>0</c:v>
+                  <c:v>1.7953494471509861</c:v>
                 </c:pt>
                 <c:pt idx="23">
-                  <c:v>0</c:v>
+                  <c:v>0.66240942939085234</c:v>
                 </c:pt>
                 <c:pt idx="24">
-                  <c:v>0</c:v>
+                  <c:v>0.27714759903786063</c:v>
                 </c:pt>
                 <c:pt idx="25">
-                  <c:v>0</c:v>
+                  <c:v>0.23872194191046633</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -23598,6 +23643,8 @@
     <col min="14" max="14" width="18.54296875" bestFit="1" customWidth="1"/>
     <col min="16" max="16" width="18.08984375" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="25.1796875" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="24.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:37" x14ac:dyDescent="0.35">
@@ -23791,6 +23838,45 @@
       <c r="O6">
         <v>15.651999999999999</v>
       </c>
+      <c r="P6">
+        <v>14.798</v>
+      </c>
+      <c r="Q6">
+        <v>17.056000000000001</v>
+      </c>
+      <c r="R6">
+        <v>18.266999999999999</v>
+      </c>
+      <c r="S6">
+        <v>21.821999999999999</v>
+      </c>
+      <c r="T6">
+        <v>22.454000000000001</v>
+      </c>
+      <c r="U6">
+        <v>18.934000000000001</v>
+      </c>
+      <c r="V6">
+        <v>16.04</v>
+      </c>
+      <c r="W6">
+        <v>13.116</v>
+      </c>
+      <c r="X6">
+        <v>9.7759999999999998</v>
+      </c>
+      <c r="Y6">
+        <v>7.2060000000000004</v>
+      </c>
+      <c r="Z6">
+        <v>2.6560000000000001</v>
+      </c>
+      <c r="AA6">
+        <v>1.1100000000000001</v>
+      </c>
+      <c r="AB6">
+        <v>0.95599999999999996</v>
+      </c>
     </row>
     <row r="7" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A7" s="3"/>
@@ -23836,6 +23922,45 @@
       <c r="O7">
         <v>-55.795000000000002</v>
       </c>
+      <c r="P7">
+        <v>-60.820999999999998</v>
+      </c>
+      <c r="Q7">
+        <v>-67.641999999999996</v>
+      </c>
+      <c r="R7">
+        <v>-73.385999999999996</v>
+      </c>
+      <c r="S7">
+        <v>-84.156000000000006</v>
+      </c>
+      <c r="T7">
+        <v>-90.259</v>
+      </c>
+      <c r="U7">
+        <v>-75.180999999999997</v>
+      </c>
+      <c r="V7">
+        <v>-65.846999999999994</v>
+      </c>
+      <c r="W7">
+        <v>-51.487000000000002</v>
+      </c>
+      <c r="X7">
+        <v>-33.896000000000001</v>
+      </c>
+      <c r="Y7">
+        <v>-17.023</v>
+      </c>
+      <c r="Z7">
+        <v>-4.0990000000000002</v>
+      </c>
+      <c r="AA7">
+        <v>6.3120000000000003</v>
+      </c>
+      <c r="AB7">
+        <v>16.004999999999999</v>
+      </c>
     </row>
     <row r="8" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A8" s="3"/>
@@ -23881,6 +24006,45 @@
       <c r="O8">
         <v>622.85</v>
       </c>
+      <c r="P8">
+        <v>623.60699999999997</v>
+      </c>
+      <c r="Q8">
+        <v>623.60699999999997</v>
+      </c>
+      <c r="R8">
+        <v>622.096</v>
+      </c>
+      <c r="S8">
+        <v>620.57899999999995</v>
+      </c>
+      <c r="T8">
+        <v>622.85</v>
+      </c>
+      <c r="U8">
+        <v>623.85</v>
+      </c>
+      <c r="V8">
+        <v>622.85</v>
+      </c>
+      <c r="W8">
+        <v>621.33600000000001</v>
+      </c>
+      <c r="X8">
+        <v>622.09299999999996</v>
+      </c>
+      <c r="Y8">
+        <v>623.60699999999997</v>
+      </c>
+      <c r="Z8">
+        <v>622.85</v>
+      </c>
+      <c r="AA8">
+        <v>622.09299999999996</v>
+      </c>
+      <c r="AB8">
+        <v>621.33600000000001</v>
+      </c>
     </row>
     <row r="9" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A9" s="11" t="s">
@@ -23928,19 +24092,45 @@
       <c r="O9" s="1">
         <v>75</v>
       </c>
-      <c r="P9" s="1"/>
-      <c r="Q9" s="1"/>
-      <c r="R9" s="1"/>
-      <c r="S9" s="1"/>
-      <c r="T9" s="1"/>
-      <c r="U9" s="1"/>
-      <c r="V9" s="1"/>
-      <c r="W9" s="1"/>
-      <c r="X9" s="1"/>
-      <c r="Y9" s="1"/>
-      <c r="Z9" s="1"/>
-      <c r="AA9" s="1"/>
-      <c r="AB9" s="1"/>
+      <c r="P9" s="1">
+        <v>74</v>
+      </c>
+      <c r="Q9" s="1">
+        <v>74</v>
+      </c>
+      <c r="R9" s="1">
+        <v>73</v>
+      </c>
+      <c r="S9" s="1">
+        <v>74</v>
+      </c>
+      <c r="T9" s="1">
+        <v>75</v>
+      </c>
+      <c r="U9" s="1">
+        <v>74</v>
+      </c>
+      <c r="V9" s="1">
+        <v>74</v>
+      </c>
+      <c r="W9" s="1">
+        <v>76</v>
+      </c>
+      <c r="X9" s="1">
+        <v>79</v>
+      </c>
+      <c r="Y9" s="1">
+        <v>81</v>
+      </c>
+      <c r="Z9" s="1">
+        <v>82</v>
+      </c>
+      <c r="AA9" s="1">
+        <v>84</v>
+      </c>
+      <c r="AB9" s="1">
+        <v>85</v>
+      </c>
       <c r="AC9" s="1"/>
       <c r="AD9" s="1"/>
       <c r="AE9" s="1"/>
@@ -23959,41 +24149,80 @@
       <c r="C10" s="16">
         <v>404</v>
       </c>
-      <c r="D10" s="33">
+      <c r="D10">
         <v>398</v>
       </c>
-      <c r="E10" s="33">
+      <c r="E10">
         <v>393</v>
       </c>
-      <c r="F10" s="33">
+      <c r="F10">
         <v>393</v>
       </c>
-      <c r="G10" s="33">
+      <c r="G10">
         <v>390</v>
       </c>
-      <c r="H10" s="33">
+      <c r="H10">
         <v>394</v>
       </c>
-      <c r="I10" s="33">
+      <c r="I10">
         <v>397</v>
       </c>
-      <c r="J10" s="33">
+      <c r="J10">
         <v>399</v>
       </c>
-      <c r="K10" s="33">
+      <c r="K10">
         <v>400</v>
       </c>
-      <c r="L10" s="33">
+      <c r="L10">
         <v>404</v>
       </c>
-      <c r="M10" s="33">
+      <c r="M10">
         <v>407</v>
       </c>
-      <c r="N10" s="33">
+      <c r="N10">
         <v>410</v>
       </c>
-      <c r="O10" s="33">
+      <c r="O10">
         <v>410</v>
+      </c>
+      <c r="P10" s="33">
+        <v>414</v>
+      </c>
+      <c r="Q10" s="33">
+        <v>415</v>
+      </c>
+      <c r="R10" s="33">
+        <v>416</v>
+      </c>
+      <c r="S10" s="33">
+        <v>423</v>
+      </c>
+      <c r="T10" s="33">
+        <v>424</v>
+      </c>
+      <c r="U10" s="33">
+        <v>418</v>
+      </c>
+      <c r="V10" s="33">
+        <v>417</v>
+      </c>
+      <c r="W10" s="33">
+        <v>410</v>
+      </c>
+      <c r="X10" s="33">
+        <v>404</v>
+      </c>
+      <c r="Y10" s="33">
+        <v>396</v>
+      </c>
+      <c r="Z10" s="33">
+        <v>387</v>
+      </c>
+      <c r="AA10" s="33">
+        <v>388</v>
+      </c>
+      <c r="AB10" s="33">
+        <v>387</v>
       </c>
     </row>
     <row r="11" spans="1:37" x14ac:dyDescent="0.35">
@@ -24184,6 +24413,45 @@
       <c r="O14">
         <v>30</v>
       </c>
+      <c r="P14">
+        <v>28</v>
+      </c>
+      <c r="Q14">
+        <v>28</v>
+      </c>
+      <c r="R14">
+        <v>28</v>
+      </c>
+      <c r="S14">
+        <v>28</v>
+      </c>
+      <c r="T14">
+        <v>27</v>
+      </c>
+      <c r="U14">
+        <v>30</v>
+      </c>
+      <c r="V14">
+        <v>29</v>
+      </c>
+      <c r="W14">
+        <v>33</v>
+      </c>
+      <c r="X14">
+        <v>37</v>
+      </c>
+      <c r="Y14">
+        <v>44</v>
+      </c>
+      <c r="Z14">
+        <v>50</v>
+      </c>
+      <c r="AA14">
+        <v>59</v>
+      </c>
+      <c r="AB14">
+        <v>72</v>
+      </c>
     </row>
     <row r="15" spans="1:37" x14ac:dyDescent="0.35">
       <c r="A15" s="13"/>
@@ -24285,138 +24553,144 @@
       </c>
       <c r="P16" s="16">
         <f t="shared" si="0"/>
+        <v>3.6291506505175044</v>
+      </c>
+      <c r="Q16" s="16">
+        <f t="shared" si="0"/>
+        <v>4.1829161707816302</v>
+      </c>
+      <c r="R16" s="16">
+        <f t="shared" si="0"/>
+        <v>4.4642414453654187</v>
+      </c>
+      <c r="S16" s="16">
+        <f t="shared" si="0"/>
+        <v>5.3517587170964296</v>
+      </c>
+      <c r="T16" s="16">
+        <f t="shared" si="0"/>
+        <v>5.5243356546689117</v>
+      </c>
+      <c r="U16" s="16">
+        <f t="shared" si="0"/>
+        <v>4.6434882022501975</v>
+      </c>
+      <c r="V16" s="16">
+        <f>V6*SIN(RADIANS(V9+5.15))*V13/1000</f>
+        <v>3.9337462112650874</v>
+      </c>
+      <c r="W16" s="16">
+        <f t="shared" si="0"/>
+        <v>3.2362035092330919</v>
+      </c>
+      <c r="X16" s="16">
+        <f t="shared" si="0"/>
+        <v>2.4284517189520791</v>
+      </c>
+      <c r="Y16" s="16">
+        <f t="shared" si="0"/>
+        <v>1.7953494471509861</v>
+      </c>
+      <c r="Z16" s="16">
+        <f t="shared" si="0"/>
+        <v>0.66240942939085234</v>
+      </c>
+      <c r="AA16" s="16">
+        <f t="shared" si="0"/>
+        <v>0.27714759903786063</v>
+      </c>
+      <c r="AB16" s="16">
+        <f t="shared" si="0"/>
+        <v>0.23872194191046633</v>
+      </c>
+      <c r="AC16" s="16">
+        <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="Q16" s="16">
+      <c r="AD16" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="R16" s="16">
+      <c r="AE16" s="16">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="S16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="T16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="U16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="V16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="W16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="X16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Y16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="Z16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AA16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AB16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AC16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AD16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="AE16" s="16">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17" spans="1:15" x14ac:dyDescent="0.35">
+    </row>
+    <row r="17" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A17" s="3"/>
       <c r="B17" s="3"/>
       <c r="N17" s="3"/>
       <c r="O17" s="3"/>
-    </row>
-    <row r="18" spans="1:15" x14ac:dyDescent="0.35">
+      <c r="S17" t="s">
+        <v>85</v>
+      </c>
+      <c r="T17" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="18" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A18" s="3"/>
       <c r="B18" t="s">
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A19" s="3"/>
       <c r="B19" s="3"/>
     </row>
-    <row r="20" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A20" s="3"/>
       <c r="B20" s="3"/>
     </row>
-    <row r="21" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A21" s="3"/>
       <c r="B21" s="21" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="22" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A22" s="3"/>
       <c r="B22" s="3"/>
     </row>
-    <row r="23" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A23" s="3"/>
       <c r="B23" s="3"/>
     </row>
-    <row r="24" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A24" s="3"/>
       <c r="B24" s="3"/>
     </row>
-    <row r="25" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A25" s="3"/>
       <c r="B25" s="3"/>
     </row>
-    <row r="26" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A26" s="3"/>
       <c r="B26" s="3"/>
     </row>
-    <row r="27" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A27" s="3"/>
       <c r="B27" s="29" t="s">
         <v>69</v>
       </c>
     </row>
-    <row r="28" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A28" s="3"/>
       <c r="B28" s="3"/>
     </row>
-    <row r="29" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A29" s="3"/>
       <c r="B29" s="3"/>
     </row>
-    <row r="30" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A30" s="3"/>
       <c r="B30" s="3"/>
     </row>
-    <row r="31" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A31" s="3"/>
       <c r="B31" s="3"/>
     </row>
-    <row r="32" spans="1:15" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:20" x14ac:dyDescent="0.35">
       <c r="A32" s="3"/>
       <c r="B32" s="3"/>
     </row>

</xml_diff>

<commit_message>
prepping minimizeFlxPin10mm to run with new data
removed bad tests from 46cm length. Added new data from 42cm length. This run will include the 48cm length tests but I will run the optimizer on a second machine where I only change allBPA to allBPA = [2, 3, 4, 5]
</commit_message>
<xml_diff>
--- a/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
+++ b/Testing_Data/2026_06_Festo/Results_table_10mm_pinned.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ben\Documents\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\GitHub\Bipedal_Robot\Testing_Data\2026_06_Festo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0054F3F2-613A-47F6-A79F-5F8B4D31CCDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10268781-4083-43C9-B151-833620A4857D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" firstSheet="13" activeTab="18" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
+    <workbookView xWindow="0" yWindow="1044" windowWidth="21600" windowHeight="11292" firstSheet="15" activeTab="18" xr2:uid="{FDAF32CB-2BA8-47E2-927E-3C1E6066A0C3}"/>
   </bookViews>
   <sheets>
     <sheet name="ExtTest10mm_1" sheetId="9" r:id="rId1"/>
@@ -417,7 +417,6 @@
     <author>tc={D38AB9F1-0008-44E2-9AA2-442694BB58A1}</author>
     <author>tc={8BAEE42B-9536-417D-B6B2-DB5320F80125}</author>
     <author>tc={D29CCFA0-C50E-48A0-9F07-9CBB4F001241}</author>
-    <author>tc={E616D17E-2271-4A96-95EA-0FDB020E98C3}</author>
   </authors>
   <commentList>
     <comment ref="C2" authorId="0" shapeId="0" xr:uid="{F2916077-4F60-4815-AACB-36F540965802}">
@@ -433,7 +432,9 @@
         <t>[Threaded comment]
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
-    Recheck after test</t>
+    Recheck after test
+Reply:
+    Was 387 then reduced to 384 and then 381 after a while.</t>
       </text>
     </comment>
     <comment ref="D3" authorId="2" shapeId="0" xr:uid="{8BAEE42B-9536-417D-B6B2-DB5320F80125}">
@@ -450,14 +451,6 @@
 Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
 Comment:
     Kmax</t>
-      </text>
-    </comment>
-    <comment ref="C4" authorId="4" shapeId="0" xr:uid="{E616D17E-2271-4A96-95EA-0FDB020E98C3}">
-      <text>
-        <t>[Threaded comment]
-Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
-Comment:
-    Initially measured 30 mm but noticed it was actually 35 mm around data reading 6</t>
       </text>
     </comment>
   </commentList>
@@ -24769,14 +24762,14 @@
   <threadedComment ref="C3" dT="2026-07-18T06:57:43.54" personId="{10A700E7-E0AC-4B04-B751-E14560120F23}" id="{D38AB9F1-0008-44E2-9AA2-442694BB58A1}">
     <text>Recheck after test</text>
   </threadedComment>
+  <threadedComment ref="C3" dT="2026-08-16T20:19:16.56" personId="{10A700E7-E0AC-4B04-B751-E14560120F23}" id="{2B101A1F-792E-4EA0-B36B-F4124522D90F}" parentId="{D38AB9F1-0008-44E2-9AA2-442694BB58A1}">
+    <text>Was 387 then reduced to 384 and then 381 after a while.</text>
+  </threadedComment>
   <threadedComment ref="D3" dT="2026-07-17T08:55:32.82" personId="{10A700E7-E0AC-4B04-B751-E14560120F23}" id="{8BAEE42B-9536-417D-B6B2-DB5320F80125}">
     <text>Max contracted length normalized by resting length</text>
   </threadedComment>
   <threadedComment ref="E3" dT="2026-07-17T08:54:37.64" personId="{10A700E7-E0AC-4B04-B751-E14560120F23}" id="{D29CCFA0-C50E-48A0-9F07-9CBB4F001241}">
     <text>Kmax</text>
-  </threadedComment>
-  <threadedComment ref="C4" dT="2026-07-18T06:57:17.11" personId="{10A700E7-E0AC-4B04-B751-E14560120F23}" id="{E616D17E-2271-4A96-95EA-0FDB020E98C3}">
-    <text>Initially measured 30 mm but noticed it was actually 35 mm around data reading 6</text>
   </threadedComment>
 </ThreadedComments>
 </file>
@@ -33774,15 +33767,15 @@
       </c>
       <c r="B3" s="3"/>
       <c r="C3">
-        <v>387</v>
+        <v>381</v>
       </c>
       <c r="D3">
         <f>(C3/C2)</f>
-        <v>0.84682713347921224</v>
+        <v>0.83369803063457326</v>
       </c>
       <c r="E3">
         <f>1-D3</f>
-        <v>0.15317286652078776</v>
+        <v>0.16630196936542674</v>
       </c>
     </row>
     <row r="4" spans="1:37" x14ac:dyDescent="0.3">

</xml_diff>